<commit_message>
docs(ae2): cuerpo del informe en presente (Art. 21) y Resolucion 97/23 citada en el texto
Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/AE2/20261005_CatalogoRequisitos_ThiagoLeal_v3.xlsx
+++ b/docs/AE2/20261005_CatalogoRequisitos_ThiagoLeal_v3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ec7050e6095d21e4/Escritorio/Tesis/devolucion_AE2/build/_salida/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_EE7F689BE173CCD170B55FC9E497D0D422539C45" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_0EB9F3FBB3D4F05D31A35FC9E4875BD76E728DAD" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -256,7 +256,7 @@
     <t>Automatiza la liquidación y elimina las sumas manuales de tiempos de estadía.</t>
   </si>
   <si>
-    <t>Condición inicial: tarifa Estándar vigente ($8.000 por 120 min y $2.500 por cada fracción de 30 min o porción, sin tolerancia) y un turno En Curso. Acción: pedir el resumen del turno a los 120, 121, 150 y 151 min. Resultado: sobreturno de $0, $2.500, $2.500 y $5.000; total = tarifa base + sobreturno + consumos (RN-DER-01 y RN-DER-02). La gerencia aprobó los importes de la tarifa en el acta del 06/10/2026; el acta del 23/09 había aprobado la regla.</t>
+    <t>Condición inicial: tarifa Estándar vigente ($8.000 por 120 min y $2.500 por cada fracción de 30 min o porción, sin tolerancia) y un turno En Curso. Acción: pedir el resumen del turno a los 120, 121, 150 y 151 min. Resultado: sobreturno de $0, $2.500, $2.500 y $5.000; total = tarifa base + sobreturno + consumos (RN-DER-01 y RN-DER-02). La gerencia aprueba los importes de la tarifa en el acta del 06/10/2026; el acta del 23/09 aprueba la regla.</t>
   </si>
   <si>
     <t>H-05, H-07, H-16 · Acta 23/09</t>
@@ -457,7 +457,7 @@
     <t>El cobro debe resolverse en un paso, sin demorar al cliente en la salida (H-08).</t>
   </si>
   <si>
-    <t>Condición inicial: API en el entorno de despliegue con 5 peticiones concurrentes de apertura y 5 de cobro. Acción: repetir 20 veces y medir la latencia. Resultado: el percentil 95 es de 800 ms o menos. La gerencia aprobó el umbral en el acta del 06/10/2026.</t>
+    <t>Condición inicial: API en el entorno de despliegue con 5 peticiones concurrentes de apertura y 5 de cobro. Acción: repetir 20 veces y medir la latencia. Resultado: el percentil 95 es de 800 ms o menos. La gerencia aprueba el umbral en el acta del 06/10/2026.</t>
   </si>
   <si>
     <t>H-02, H-08, H-14 · Acta 23/09</t>
@@ -493,7 +493,7 @@
     <t>El cierre ciego necesita saber a quién atribuir un faltante (RF-09) y la AE1 exige delimitar responsabilidades (H-06).</t>
   </si>
   <si>
-    <t>Condición inicial: dos conserjes con credenciales propias. Acción: un conserje inicia sesión y ejecuta una apertura y un cobro; desde la consola del navegador se ejecuta document.cookie. Resultado: el token JWT no es visible (cookie httpOnly), el turno y el pago registran el identificador de ese operador y una petición sin token responde 401. La gerencia aprobó el requisito en el acta del 06/10/2026; el mecanismo se decide en el prototipo v2.</t>
+    <t>Condición inicial: dos conserjes con credenciales propias. Acción: un conserje inicia sesión y ejecuta una apertura y un cobro; desde la consola del navegador se ejecuta document.cookie. Resultado: el token JWT no es visible (cookie httpOnly), el turno y el pago registran el identificador de ese operador y una petición sin token responde 401. La gerencia aprueba el requisito en el acta del 06/10/2026; el mecanismo se decide en el prototipo v2.</t>
   </si>
   <si>
     <t>H-06, H-17 · Acta 23/09</t>
@@ -508,7 +508,7 @@
     <t>Usabilidad</t>
   </si>
   <si>
-    <t>Debe operar en la terminal de la ventanilla. La gerencia aprobó el requisito en el acta del 06/10/2026, pero la resolución real de ese monitor no se informó; la interfaz se diseña para 1366 × 768 px como mínimo.</t>
+    <t>Debe operar en la terminal de la ventanilla. La gerencia aprueba el requisito en el acta del 06/10/2026, pero la resolución real de ese monitor no se informa; la interfaz se diseña para 1366 × 768 px como mínimo.</t>
   </si>
   <si>
     <t>Condición inicial: navegador a 1366 × 768 px. Acción: recorrer apertura, consumo y cobro. Resultado: no aparece barra de desplazamiento horizontal y cada control tiene un área de clic de al menos 44 × 44 px, comprobada con las herramientas del navegador.</t>
@@ -556,7 +556,7 @@
     <t>La patente de un turno se elimina dentro de las 24 h posteriores a su cierre.</t>
   </si>
   <si>
-    <t>La patente identifica de forma indirecta al titular del vehículo; se conserva mientras el vehículo está en el motel y luego se elimina (Ley 25.326, art. 4, inc. 7). La gerencia aprobó las 24 h en el acta del 06/10/2026 y declaró que necesita la patente por razones de seguridad; informó que no hay indicación del asesor legal.</t>
+    <t>La patente identifica de forma indirecta al titular del vehículo; se conserva mientras el vehículo está en el motel y luego se elimina (Ley 25.326, art. 4, inc. 7). La gerencia aprueba las 24 h en el acta del 06/10/2026, declara que necesita la patente por razones de seguridad e informa que no hay indicación del asesor legal.</t>
   </si>
   <si>
     <t>Condición inicial: turno FINALIZADO con patente AE987CD, cerrado hace más de 24 h. Acción: ejecutar la depuración y consultar los turnos cerrados y la tabla de estadía activa. Resultado: ninguna patente de un turno cerrado hace más de 24 h permanece almacenada (la consulta devuelve 0 filas) y los importes del turno quedan intactos, sin deshabilitar los triggers de inmutabilidad.</t>
@@ -574,7 +574,7 @@
     <t>Es la decisión de la AE1 para las intermitencias de internet (H-09); reemplaza la idea de persistencia local en caché, que no se sostiene con el servidor en la nube.</t>
   </si>
   <si>
-    <t>Condición inicial: tres turnos En Curso. Acción: cortar la conexión del navegador durante 10 min y restablecerla. Resultado: en 5 s o menos la grilla muestra los tres turnos con los minutos calculados por el servidor (diferencia de 1 min o menos respecto de su reloj), sin turnos perdidos ni duplicados. Durante el corte no se pueden abrir ni cobrar turnos; el procedimiento de contingencia manual no se definió en la sesión del 06/10/2026; el autor propone anotar los turnos en papel y cargarlos al volver la conexión.</t>
+    <t>Condición inicial: tres turnos En Curso. Acción: cortar la conexión del navegador durante 10 min y restablecerla. Resultado: en 5 s o menos la grilla muestra los tres turnos con los minutos calculados por el servidor (diferencia de 1 min o menos respecto de su reloj), sin turnos perdidos ni duplicados. Durante el corte no se pueden abrir ni cobrar turnos; el procedimiento de contingencia manual no se define en la sesión del 06/10/2026; el autor propone anotar los turnos en papel y cargarlos al volver la conexión.</t>
   </si>
   <si>
     <t>Matriz de trazabilidad · hallazgo de la AE1 → requisito</t>
@@ -604,7 +604,7 @@
     <t>H-01</t>
   </si>
   <si>
-    <t>13 habitaciones, 3 guardias diarias y unos 30 turnos por día hábil (lunes a jueves) y unos 40 en fin de semana (viernes a domingo). La AE1 original informaba 20 a 30 y 40 a 50; rige lo que la gerencia dijo en la entrevista.</t>
+    <t>13 habitaciones, 3 guardias diarias y unos 30 turnos por día hábil (lunes a jueves) y unos 40 en fin de semana (viernes a domingo). La AE1 original informa 20 a 30 y 40 a 50; rige lo que la gerencia dice en la entrevista.</t>
   </si>
   <si>
     <t>AE1 · II.3 (v2) y entrevista, pág. 1</t>
@@ -718,7 +718,7 @@
     <t>H-11</t>
   </si>
   <si>
-    <t>El personal de maestranza y limpieza quedó fuera del relevamiento; los tiempos de limpieza son estimaciones indirectas de conserjería.</t>
+    <t>El personal de maestranza y limpieza queda fuera del relevamiento; los tiempos de limpieza son estimaciones indirectas de conserjería.</t>
   </si>
   <si>
     <t>AE1 · II.2 y II.6 (limitaciones)</t>
@@ -1384,7 +1384,7 @@
     <t>RF-08, RF-09, RNF-02, RNF-04, RNF-08 (5 Must) y RNF-07</t>
   </si>
   <si>
-    <t>Prototipo v2: cierre ciego con pruebas automáticas. La retención de la patente (RNF-08) y el rol de aplicación se adelantaron a la v1.2 (05/10/2026).</t>
+    <t>Prototipo v2: cierre ciego con pruebas automáticas. La retención de la patente (RNF-08) y el rol de aplicación se adelantan a la v1.2 (05/10/2026).</t>
   </si>
   <si>
     <t>02/11/2026</t>
@@ -9598,7 +9598,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="66" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" ht="54" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="13">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
docs(ae2): resolucion del monitor de la ventanilla (1366 x 768) relevada por el autor
Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/AE2/20261005_CatalogoRequisitos_ThiagoLeal_v3.xlsx
+++ b/docs/AE2/20261005_CatalogoRequisitos_ThiagoLeal_v3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ec7050e6095d21e4/Escritorio/Tesis/devolucion_AE2/build/_salida/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_0EB9F3FBB3D4F05D31A35FC9E4875BD76E728DAD" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_0EB9574B43C51080F1AF5F29E4BA83D0C872A235" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -508,13 +508,13 @@
     <t>Usabilidad</t>
   </si>
   <si>
-    <t>Debe operar en la terminal de la ventanilla. La gerencia aprueba el requisito en el acta del 06/10/2026, pero la resolución real de ese monitor no se informa; la interfaz se diseña para 1366 × 768 px como mínimo.</t>
+    <t>Debe operar en la terminal de la ventanilla. La gerencia aprueba el requisito en el acta del 06/10/2026 y el autor relevó en el local que ese monitor es de 1366 × 768 px.</t>
   </si>
   <si>
     <t>Condición inicial: navegador a 1366 × 768 px. Acción: recorrer apertura, consumo y cobro. Resultado: no aparece barra de desplazamiento horizontal y cada control tiene un área de clic de al menos 44 × 44 px, comprobada con las herramientas del navegador.</t>
   </si>
   <si>
-    <t>Sin hallazgo: relevar y fechar la resolución del monitor de la ventanilla · Acta 23/09</t>
+    <t>Sin hallazgo: relevamiento del autor en el local (monitor de 1366 × 768 px) · Acta 23/09</t>
   </si>
   <si>
     <t>RNF-06</t>
@@ -1645,7 +1645,7 @@
     <t>equipo</t>
   </si>
   <si>
-    <t>Equipo del motel; sin costo para el proyecto. Resolución real del monitor no informada; se diseña para 1366 × 768 px (RNF-05).</t>
+    <t>Equipo del motel; sin costo para el proyecto. Monitor de 1366 × 768 px, relevado por el autor (RNF-05).</t>
   </si>
   <si>
     <t>Terminal POSNET</t>
@@ -1987,7 +1987,7 @@
     <t>Monitor de 1366 × 768 en la ventanilla</t>
   </si>
   <si>
-    <t>No informada por la gerencia; RNF-05 aprobado en el acta del 06/10/2026.</t>
+    <t>Relevada por el autor en el local: 1366 × 768 px; RNF-05 aprobado en el acta del 06/10/2026.</t>
   </si>
   <si>
     <t>Parálisis ante cortes de conectividad</t>
@@ -3773,7 +3773,7 @@
         <v>Fila completa</v>
       </c>
     </row>
-    <row r="22" spans="1:12" ht="102" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" ht="78" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="12" t="s">
         <v>139</v>
       </c>
@@ -10761,7 +10761,7 @@
         <v>517</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="12" t="s">
         <v>518</v>
       </c>

</xml_diff>